<commit_message>
Adding new content from stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="252">
   <si>
     <t xml:space="preserve">Project:</t>
   </si>
@@ -544,7 +544,7 @@
     <t xml:space="preserve">667-ERA-3AEB682V</t>
   </si>
   <si>
-    <t xml:space="preserve">R4,R20,R21,R23,R24,R30</t>
+    <t xml:space="preserve">R4,R20,R21,R23,R24,R30,R9,R10,R11,R15,R16,R17</t>
   </si>
   <si>
     <t xml:space="preserve">RC060310K2075AAA</t>
@@ -580,12 +580,6 @@
     <t xml:space="preserve">603-AC1210JR-071K2L</t>
   </si>
   <si>
-    <t xml:space="preserve">R9,R10,R11,R15,R16,R17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC06010K2075AAA</t>
-  </si>
-  <si>
     <t xml:space="preserve">R18</t>
   </si>
   <si>
@@ -700,7 +694,7 @@
     <t xml:space="preserve">P1012202501-PCB-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Jumper for J1</t>
+    <t xml:space="preserve">Jumper for J1, J2, and J3</t>
   </si>
   <si>
     <t xml:space="preserve">JMP2POS1ROW254</t>
@@ -815,7 +809,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -830,26 +824,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC9211E"/>
-        <bgColor rgb="FFFF3838"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF3838"/>
-        <bgColor rgb="FFFF4000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF5429"/>
-        <bgColor rgb="FFFF4000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF4000"/>
-        <bgColor rgb="FFFF3838"/>
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008000"/>
       </patternFill>
     </fill>
   </fills>
@@ -894,7 +870,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -927,7 +903,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -935,55 +919,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1000,7 +940,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF3838"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1019,7 +959,7 @@
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF4000"/>
+      <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
@@ -1043,14 +983,14 @@
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF5429"/>
+      <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFC9211E"/>
+      <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -1170,10 +1110,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.77"/>
@@ -1203,15 +1143,15 @@
         <v>2</v>
       </c>
       <c r="I1" s="2" t="n">
-        <f aca="false">SUM(I6:I62)</f>
-        <v>77.05</v>
+        <f aca="false">SUM(I6:I61)</f>
+        <v>77.51</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="K1" s="2" t="n">
-        <f aca="false">SUM(K6:K57)</f>
-        <v>26.047</v>
+        <f aca="false">SUM(K6:K56)</f>
+        <v>26.269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1273,7 +1213,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>21</v>
       </c>
@@ -1292,20 +1232,20 @@
       <c r="F6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="9" t="n">
         <v>0.22</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="9" t="n">
         <f aca="false">B6*H6</f>
         <v>0.88</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="9" t="n">
         <v>0.068</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="9" t="n">
         <f aca="false">B6*J6</f>
         <v>0.272</v>
       </c>
@@ -1315,7 +1255,7 @@
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
     </row>
-    <row r="7" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
@@ -1334,20 +1274,20 @@
       <c r="F7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="9" t="n">
         <f aca="false">B7*H7</f>
         <v>1.1</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="9" t="n">
         <v>0.012</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="9" t="n">
         <f aca="false">B7*J7</f>
         <v>0.132</v>
       </c>
@@ -1357,7 +1297,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
     </row>
-    <row r="8" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
         <v>32</v>
       </c>
@@ -1376,20 +1316,20 @@
       <c r="F8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>0.6</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="9" t="n">
         <f aca="false">B8*H8</f>
         <v>2.4</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="9" t="n">
         <v>0.187</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K8" s="9" t="n">
         <f aca="false">B8*J8</f>
         <v>0.748</v>
       </c>
@@ -1399,7 +1339,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
     </row>
-    <row r="9" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>37</v>
       </c>
@@ -1418,20 +1358,20 @@
       <c r="F9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="9" t="n">
         <f aca="false">B9*H9</f>
         <v>0.5</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="9" t="n">
         <v>0.023</v>
       </c>
-      <c r="K9" s="8" t="n">
+      <c r="K9" s="9" t="n">
         <f aca="false">B9*J9</f>
         <v>0.115</v>
       </c>
@@ -1441,7 +1381,7 @@
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
     </row>
-    <row r="10" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>42</v>
       </c>
@@ -1460,20 +1400,20 @@
       <c r="F10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="9" t="n">
         <f aca="false">B10*H10</f>
         <v>0.2</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="9" t="n">
         <v>0.043</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K10" s="9" t="n">
         <f aca="false">B10*J10</f>
         <v>0.086</v>
       </c>
@@ -1483,7 +1423,7 @@
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
     </row>
-    <row r="11" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>46</v>
       </c>
@@ -1502,20 +1442,20 @@
       <c r="F11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <v>1.49</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="9" t="n">
         <f aca="false">B11*H11</f>
         <v>1.49</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J11" s="9" t="n">
         <v>0.472</v>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="K11" s="9" t="n">
         <f aca="false">B11*J11</f>
         <v>0.472</v>
       </c>
@@ -1525,7 +1465,7 @@
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
     </row>
-    <row r="12" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>51</v>
       </c>
@@ -1544,20 +1484,20 @@
       <c r="F12" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="9" t="n">
         <f aca="false">B12*H12</f>
         <v>0.1</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="9" t="n">
         <v>0.019</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="K12" s="9" t="n">
         <f aca="false">B12*J12</f>
         <v>0.019</v>
       </c>
@@ -1567,7 +1507,7 @@
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
     </row>
-    <row r="13" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>55</v>
       </c>
@@ -1586,20 +1526,20 @@
       <c r="F13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="9" t="n">
         <f aca="false">B13*H13</f>
         <v>0.15</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="9" t="n">
         <v>0.035</v>
       </c>
-      <c r="K13" s="8" t="n">
+      <c r="K13" s="9" t="n">
         <f aca="false">B13*J13</f>
         <v>0.035</v>
       </c>
@@ -1609,133 +1549,133 @@
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="9" t="n">
         <v>0.33</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="9" t="n">
         <f aca="false">B14*H14</f>
         <v>0.33</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J14" s="9" t="n">
         <v>0.128</v>
       </c>
-      <c r="K14" s="6" t="n">
+      <c r="K14" s="9" t="n">
         <f aca="false">B14*J14</f>
         <v>0.128</v>
       </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+    </row>
+    <row r="15" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="4" t="s">
+      <c r="F15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="9" t="n">
         <v>0.48</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="9" t="n">
         <f aca="false">B15*H15</f>
         <v>0.48</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="9" t="n">
         <v>0.189</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="K15" s="9" t="n">
         <f aca="false">B15*J15</f>
         <v>0.189</v>
       </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+    </row>
+    <row r="16" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="4" t="s">
+      <c r="F16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="9" t="n">
         <v>0.62</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="9" t="n">
         <f aca="false">B16*H16</f>
         <v>1.86</v>
       </c>
-      <c r="J16" s="6" t="n">
+      <c r="J16" s="9" t="n">
         <v>0.246</v>
       </c>
-      <c r="K16" s="6" t="n">
+      <c r="K16" s="9" t="n">
         <f aca="false">B16*J16</f>
         <v>0.738</v>
       </c>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-    </row>
-    <row r="17" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+    </row>
+    <row r="17" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>73</v>
       </c>
@@ -1754,20 +1694,20 @@
       <c r="F17" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="9" t="n">
         <v>0.78</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="9" t="n">
         <f aca="false">B17*H17</f>
         <v>0.78</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J17" s="9" t="n">
         <v>0.484</v>
       </c>
-      <c r="K17" s="8" t="n">
+      <c r="K17" s="9" t="n">
         <f aca="false">B17*J17</f>
         <v>0.484</v>
       </c>
@@ -1777,49 +1717,49 @@
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="4" t="s">
+      <c r="F18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="9" t="n">
         <v>0.79</v>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I18" s="9" t="n">
         <f aca="false">B18*H18</f>
         <v>0.79</v>
       </c>
-      <c r="J18" s="6" t="n">
+      <c r="J18" s="9" t="n">
         <v>0.369</v>
       </c>
-      <c r="K18" s="6" t="n">
+      <c r="K18" s="9" t="n">
         <f aca="false">B18*J18</f>
         <v>0.369</v>
       </c>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
-    </row>
-    <row r="19" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+    </row>
+    <row r="19" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>83</v>
       </c>
@@ -1838,20 +1778,20 @@
       <c r="F19" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="9" t="n">
         <v>0.27</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="9" t="n">
         <f aca="false">B19*H19</f>
         <v>0.54</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="9" t="n">
         <v>0.049</v>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="K19" s="9" t="n">
         <f aca="false">B19*J19</f>
         <v>0.098</v>
       </c>
@@ -1861,7 +1801,7 @@
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
     </row>
-    <row r="20" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>88</v>
       </c>
@@ -1880,20 +1820,20 @@
       <c r="F20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>0.36</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="9" t="n">
         <f aca="false">B20*H20</f>
         <v>0.36</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="9" t="n">
         <v>0.076</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K20" s="9" t="n">
         <f aca="false">B20*J20</f>
         <v>0.076</v>
       </c>
@@ -1903,7 +1843,7 @@
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
     </row>
-    <row r="21" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>93</v>
       </c>
@@ -1922,20 +1862,20 @@
       <c r="F21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="9" t="n">
         <v>1.11</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="9" t="n">
         <f aca="false">B21*H21</f>
         <v>5.55</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="9" t="n">
         <v>0.343</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="K21" s="9" t="n">
         <f aca="false">B21*J21</f>
         <v>1.715</v>
       </c>
@@ -1945,7 +1885,7 @@
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
     </row>
-    <row r="22" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>98</v>
       </c>
@@ -1964,20 +1904,20 @@
       <c r="F22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="9" t="n">
         <f aca="false">B22*H22</f>
         <v>0.15</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="9" t="n">
         <v>0.045</v>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="K22" s="9" t="n">
         <f aca="false">B22*J22</f>
         <v>0.045</v>
       </c>
@@ -1987,7 +1927,7 @@
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
     </row>
-    <row r="23" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>102</v>
       </c>
@@ -2006,20 +1946,20 @@
       <c r="F23" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="9" t="n">
         <v>0.71</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="9" t="n">
         <f aca="false">B23*H23</f>
         <v>0.71</v>
       </c>
-      <c r="J23" s="8" t="n">
+      <c r="J23" s="9" t="n">
         <v>0.342</v>
       </c>
-      <c r="K23" s="8" t="n">
+      <c r="K23" s="9" t="n">
         <f aca="false">B23*J23</f>
         <v>0.342</v>
       </c>
@@ -2029,7 +1969,7 @@
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
     </row>
-    <row r="24" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
         <v>107</v>
       </c>
@@ -2048,20 +1988,20 @@
       <c r="F24" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H24" s="9" t="n">
         <v>0.71</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="9" t="n">
         <f aca="false">B24*H24</f>
         <v>0.71</v>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J24" s="9" t="n">
         <v>0.342</v>
       </c>
-      <c r="K24" s="8" t="n">
+      <c r="K24" s="9" t="n">
         <f aca="false">B24*J24</f>
         <v>0.342</v>
       </c>
@@ -2071,7 +2011,7 @@
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
     </row>
-    <row r="25" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
         <v>111</v>
       </c>
@@ -2090,20 +2030,20 @@
       <c r="F25" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="9" t="n">
         <v>6.71</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="9" t="n">
         <f aca="false">B25*H25</f>
         <v>6.71</v>
       </c>
-      <c r="J25" s="8" t="n">
+      <c r="J25" s="9" t="n">
         <v>3.98</v>
       </c>
-      <c r="K25" s="8" t="n">
+      <c r="K25" s="9" t="n">
         <f aca="false">B25*J25</f>
         <v>3.98</v>
       </c>
@@ -2113,7 +2053,7 @@
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
     </row>
-    <row r="26" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
         <v>115</v>
       </c>
@@ -2132,20 +2072,20 @@
       <c r="F26" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="9" t="n">
         <v>0.81</v>
       </c>
-      <c r="I26" s="8" t="n">
+      <c r="I26" s="9" t="n">
         <f aca="false">B26*H26</f>
         <v>0.81</v>
       </c>
-      <c r="J26" s="8" t="n">
+      <c r="J26" s="9" t="n">
         <v>0.38</v>
       </c>
-      <c r="K26" s="8" t="n">
+      <c r="K26" s="9" t="n">
         <f aca="false">B26*J26</f>
         <v>0.38</v>
       </c>
@@ -2163,7 +2103,7 @@
       </c>
       <c r="P26" s="7"/>
     </row>
-    <row r="27" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
         <v>122</v>
       </c>
@@ -2182,20 +2122,20 @@
       <c r="F27" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="9" t="n">
         <v>3.55</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="9" t="n">
         <f aca="false">B27*H27</f>
         <v>3.55</v>
       </c>
-      <c r="J27" s="8" t="n">
+      <c r="J27" s="9" t="n">
         <v>1.31</v>
       </c>
-      <c r="K27" s="8" t="n">
+      <c r="K27" s="9" t="n">
         <f aca="false">B27*J27</f>
         <v>1.31</v>
       </c>
@@ -2205,7 +2145,7 @@
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
     </row>
-    <row r="28" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
         <v>127</v>
       </c>
@@ -2224,20 +2164,20 @@
       <c r="F28" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="9" t="n">
         <v>4.03</v>
       </c>
-      <c r="I28" s="8" t="n">
+      <c r="I28" s="9" t="n">
         <f aca="false">B28*H28</f>
         <v>4.03</v>
       </c>
-      <c r="J28" s="8" t="n">
+      <c r="J28" s="9" t="n">
         <v>2.4</v>
       </c>
-      <c r="K28" s="8" t="n">
+      <c r="K28" s="9" t="n">
         <f aca="false">B28*J28</f>
         <v>2.4</v>
       </c>
@@ -2247,7 +2187,7 @@
       <c r="O28" s="7"/>
       <c r="P28" s="7"/>
     </row>
-    <row r="29" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>132</v>
       </c>
@@ -2266,20 +2206,20 @@
       <c r="F29" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="9" t="n">
         <v>1.89</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="9" t="n">
         <f aca="false">B29*H29</f>
         <v>1.89</v>
       </c>
-      <c r="J29" s="8" t="n">
+      <c r="J29" s="9" t="n">
         <v>1.22</v>
       </c>
-      <c r="K29" s="8" t="n">
+      <c r="K29" s="9" t="n">
         <f aca="false">B29*J29</f>
         <v>1.22</v>
       </c>
@@ -2289,133 +2229,133 @@
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
     </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+    <row r="30" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="4" t="n">
+      <c r="B30" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G30" s="4" t="s">
+      <c r="F30" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="H30" s="6" t="n">
+      <c r="H30" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="I30" s="9" t="n">
         <f aca="false">B30*H30</f>
         <v>0.3</v>
       </c>
-      <c r="J30" s="6" t="n">
+      <c r="J30" s="9" t="n">
         <v>0.071</v>
       </c>
-      <c r="K30" s="6" t="n">
+      <c r="K30" s="9" t="n">
         <f aca="false">B30*J30</f>
         <v>0.213</v>
       </c>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
-      <c r="P30" s="4"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="L30" s="7"/>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
+    </row>
+    <row r="31" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G31" s="4" t="s">
+      <c r="F31" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="6" t="n">
+      <c r="H31" s="9" t="n">
         <v>0.17</v>
       </c>
-      <c r="I31" s="6" t="n">
+      <c r="I31" s="9" t="n">
         <f aca="false">B31*H31</f>
         <v>0.17</v>
       </c>
-      <c r="J31" s="6" t="n">
+      <c r="J31" s="9" t="n">
         <v>0.163</v>
       </c>
-      <c r="K31" s="6" t="n">
+      <c r="K31" s="9" t="n">
         <f aca="false">B31*J31</f>
         <v>0.163</v>
       </c>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
-      <c r="P31" s="4"/>
-    </row>
-    <row r="32" s="12" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
+      <c r="L31" s="7"/>
+      <c r="M31" s="7"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="7"/>
+      <c r="P31" s="7"/>
+    </row>
+    <row r="32" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="F32" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G32" s="10" t="s">
+      <c r="F32" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="H32" s="11" t="n">
+      <c r="H32" s="9" t="n">
         <v>0.33</v>
       </c>
-      <c r="I32" s="11" t="n">
+      <c r="I32" s="9" t="n">
         <f aca="false">B32*H32</f>
         <v>0.66</v>
       </c>
-      <c r="J32" s="11" t="n">
+      <c r="J32" s="9" t="n">
         <v>0.199</v>
       </c>
-      <c r="K32" s="11" t="n">
+      <c r="K32" s="9" t="n">
         <f aca="false">B32*J32</f>
         <v>0.398</v>
       </c>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-    </row>
-    <row r="33" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L32" s="7"/>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
+      <c r="O32" s="7"/>
+      <c r="P32" s="7"/>
+    </row>
+    <row r="33" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
         <v>151</v>
       </c>
@@ -2434,20 +2374,20 @@
       <c r="F33" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="G33" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="9" t="n">
         <v>0.76</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="9" t="n">
         <f aca="false">B33*H33</f>
         <v>4.56</v>
       </c>
-      <c r="J33" s="8" t="n">
+      <c r="J33" s="9" t="n">
         <v>0.303</v>
       </c>
-      <c r="K33" s="8" t="n">
+      <c r="K33" s="9" t="n">
         <f aca="false">B33*J33</f>
         <v>1.818</v>
       </c>
@@ -2457,7 +2397,7 @@
       <c r="O33" s="7"/>
       <c r="P33" s="7"/>
     </row>
-    <row r="34" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
         <v>156</v>
       </c>
@@ -2476,20 +2416,20 @@
       <c r="F34" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G34" s="7" t="s">
+      <c r="G34" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="9" t="n">
         <v>0.14</v>
       </c>
-      <c r="I34" s="8" t="n">
+      <c r="I34" s="9" t="n">
         <f aca="false">B34*H34</f>
         <v>0.14</v>
       </c>
-      <c r="J34" s="8" t="n">
+      <c r="J34" s="9" t="n">
         <v>0.42</v>
       </c>
-      <c r="K34" s="8" t="n">
+      <c r="K34" s="9" t="n">
         <f aca="false">B34*J34</f>
         <v>0.42</v>
       </c>
@@ -2499,7 +2439,7 @@
       <c r="O34" s="7"/>
       <c r="P34" s="7"/>
     </row>
-    <row r="35" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
         <v>161</v>
       </c>
@@ -2518,20 +2458,20 @@
       <c r="F35" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="G35" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="9" t="n">
         <v>0.19</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="9" t="n">
         <f aca="false">B35*H35</f>
         <v>0.38</v>
       </c>
-      <c r="J35" s="8" t="n">
+      <c r="J35" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="K35" s="8" t="n">
+      <c r="K35" s="9" t="n">
         <f aca="false">B35*J35</f>
         <v>0.03</v>
       </c>
@@ -2541,7 +2481,7 @@
       <c r="O35" s="7"/>
       <c r="P35" s="7"/>
     </row>
-    <row r="36" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>165</v>
       </c>
@@ -2560,20 +2500,20 @@
       <c r="F36" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G36" s="7" t="s">
+      <c r="G36" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I36" s="8" t="n">
+      <c r="I36" s="9" t="n">
         <f aca="false">B36*H36</f>
         <v>0.1</v>
       </c>
-      <c r="J36" s="8" t="n">
+      <c r="J36" s="9" t="n">
         <v>0.021</v>
       </c>
-      <c r="K36" s="8" t="n">
+      <c r="K36" s="9" t="n">
         <f aca="false">B36*J36</f>
         <v>0.021</v>
       </c>
@@ -2583,7 +2523,7 @@
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
     </row>
-    <row r="37" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>169</v>
       </c>
@@ -2602,20 +2542,20 @@
       <c r="F37" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G37" s="7" t="s">
+      <c r="G37" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I37" s="8" t="n">
+      <c r="I37" s="9" t="n">
         <f aca="false">B37*H37</f>
         <v>0.1</v>
       </c>
-      <c r="J37" s="8" t="n">
+      <c r="J37" s="9" t="n">
         <v>0.043</v>
       </c>
-      <c r="K37" s="8" t="n">
+      <c r="K37" s="9" t="n">
         <f aca="false">B37*J37</f>
         <v>0.043</v>
       </c>
@@ -2625,49 +2565,49 @@
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
     </row>
-    <row r="38" s="15" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
+    <row r="38" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="C38" s="13" t="s">
+      <c r="B38" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="F38" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G38" s="13" t="s">
+      <c r="F38" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="H38" s="14" t="n">
+      <c r="H38" s="9" t="n">
         <v>0.11</v>
       </c>
-      <c r="I38" s="14" t="n">
+      <c r="I38" s="9" t="n">
         <f aca="false">B38*H38</f>
-        <v>0.66</v>
-      </c>
-      <c r="J38" s="14" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J38" s="9" t="n">
         <v>0.031</v>
       </c>
-      <c r="K38" s="14" t="n">
+      <c r="K38" s="9" t="n">
         <f aca="false">B38*J38</f>
-        <v>0.186</v>
-      </c>
-      <c r="L38" s="13"/>
-      <c r="M38" s="13"/>
-      <c r="N38" s="13"/>
-      <c r="O38" s="13"/>
-      <c r="P38" s="13"/>
-    </row>
-    <row r="39" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.372</v>
+      </c>
+      <c r="L38" s="7"/>
+      <c r="M38" s="7"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
+    </row>
+    <row r="39" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>178</v>
       </c>
@@ -2686,20 +2626,20 @@
       <c r="F39" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="7" t="s">
+      <c r="G39" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="8" t="n">
+      <c r="H39" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="I39" s="8" t="n">
+      <c r="I39" s="9" t="n">
         <f aca="false">B39*H39</f>
         <v>0.1</v>
       </c>
-      <c r="J39" s="8" t="n">
+      <c r="J39" s="9" t="n">
         <v>0.013</v>
       </c>
-      <c r="K39" s="8" t="n">
+      <c r="K39" s="9" t="n">
         <f aca="false">B39*J39</f>
         <v>0.013</v>
       </c>
@@ -2709,7 +2649,7 @@
       <c r="O39" s="7"/>
       <c r="P39" s="7"/>
     </row>
-    <row r="40" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>182</v>
       </c>
@@ -2728,20 +2668,20 @@
       <c r="F40" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G40" s="7" t="s">
+      <c r="G40" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="H40" s="8" t="n">
+      <c r="H40" s="9" t="n">
         <v>0.12</v>
       </c>
-      <c r="I40" s="8" t="n">
+      <c r="I40" s="9" t="n">
         <f aca="false">B40*H40</f>
         <v>0.72</v>
       </c>
-      <c r="J40" s="8" t="n">
+      <c r="J40" s="9" t="n">
         <v>0.041</v>
       </c>
-      <c r="K40" s="8" t="n">
+      <c r="K40" s="9" t="n">
         <f aca="false">B40*J40</f>
         <v>0.246</v>
       </c>
@@ -2751,83 +2691,83 @@
       <c r="O40" s="7"/>
       <c r="P40" s="7"/>
     </row>
-    <row r="41" s="18" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="s">
+    <row r="41" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B41" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="C41" s="16" t="s">
+      <c r="B41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E41" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="F41" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="H41" s="17" t="n">
+      <c r="D41" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="H41" s="9" t="n">
         <v>0.11</v>
       </c>
-      <c r="I41" s="17" t="n">
+      <c r="I41" s="9" t="n">
         <f aca="false">B41*H41</f>
-        <v>0.66</v>
-      </c>
-      <c r="J41" s="17" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="K41" s="17" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>0.009</v>
+      </c>
+      <c r="K41" s="9" t="n">
         <f aca="false">B41*J41</f>
-        <v>0.186</v>
-      </c>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="16"/>
-      <c r="O41" s="16"/>
-      <c r="P41" s="16"/>
-    </row>
-    <row r="42" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.009</v>
+      </c>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="7"/>
+      <c r="P41" s="7"/>
+    </row>
+    <row r="42" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B42" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>90</v>
+        <v>171</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G42" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="H42" s="8" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="I42" s="8" t="n">
+      <c r="G42" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I42" s="9" t="n">
         <f aca="false">B42*H42</f>
-        <v>0.11</v>
-      </c>
-      <c r="J42" s="8" t="n">
-        <v>0.009</v>
-      </c>
-      <c r="K42" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="K42" s="9" t="n">
         <f aca="false">B42*J42</f>
-        <v>0.009</v>
+        <v>0.042</v>
       </c>
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
@@ -2835,83 +2775,83 @@
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
     </row>
-    <row r="43" s="21" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="B43" s="19" t="n">
+    <row r="43" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <f aca="false">B43*H43</f>
+        <v>0.22</v>
+      </c>
+      <c r="J43" s="9" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="K43" s="9" t="n">
+        <f aca="false">B43*J43</f>
+        <v>0.062</v>
+      </c>
+      <c r="L43" s="7"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="7"/>
+      <c r="O43" s="7"/>
+      <c r="P43" s="7"/>
+    </row>
+    <row r="44" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B44" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C43" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="D43" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="E43" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="F43" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G43" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="H43" s="20" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I43" s="20" t="n">
-        <f aca="false">B43*H43</f>
-        <v>0.1</v>
-      </c>
-      <c r="J43" s="20" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="K43" s="20" t="n">
-        <f aca="false">B43*J43</f>
-        <v>0.042</v>
-      </c>
-      <c r="L43" s="19"/>
-      <c r="M43" s="19"/>
-      <c r="N43" s="19"/>
-      <c r="O43" s="19"/>
-      <c r="P43" s="19"/>
-    </row>
-    <row r="44" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="B44" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="C44" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G44" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="H44" s="8" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="I44" s="8" t="n">
+      <c r="G44" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="I44" s="9" t="n">
         <f aca="false">B44*H44</f>
-        <v>0.22</v>
-      </c>
-      <c r="J44" s="8" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="K44" s="8" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="K44" s="9" t="n">
         <f aca="false">B44*J44</f>
-        <v>0.062</v>
+        <v>0.139</v>
       </c>
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
@@ -2919,41 +2859,41 @@
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
     </row>
-    <row r="45" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>90</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G45" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="H45" s="8" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="I45" s="8" t="n">
+      <c r="G45" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="I45" s="9" t="n">
         <f aca="false">B45*H45</f>
-        <v>0.24</v>
-      </c>
-      <c r="J45" s="8" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="K45" s="8" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="K45" s="9" t="n">
         <f aca="false">B45*J45</f>
-        <v>0.139</v>
+        <v>0.102</v>
       </c>
       <c r="L45" s="7"/>
       <c r="M45" s="7"/>
@@ -2961,41 +2901,41 @@
       <c r="O45" s="7"/>
       <c r="P45" s="7"/>
     </row>
-    <row r="46" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B46" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>90</v>
+        <v>29</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G46" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="H46" s="8" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="I46" s="8" t="n">
+      <c r="G46" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I46" s="9" t="n">
         <f aca="false">B46*H46</f>
-        <v>0.34</v>
-      </c>
-      <c r="J46" s="8" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="K46" s="8" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="J46" s="9" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="K46" s="9" t="n">
         <f aca="false">B46*J46</f>
-        <v>0.102</v>
+        <v>0.052</v>
       </c>
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
@@ -3003,41 +2943,41 @@
       <c r="O46" s="7"/>
       <c r="P46" s="7"/>
     </row>
-    <row r="47" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>29</v>
+        <v>171</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G47" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="H47" s="8" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="I47" s="8" t="n">
+      <c r="G47" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="I47" s="9" t="n">
         <f aca="false">B47*H47</f>
-        <v>0.14</v>
-      </c>
-      <c r="J47" s="8" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="K47" s="8" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="K47" s="9" t="n">
         <f aca="false">B47*J47</f>
-        <v>0.052</v>
+        <v>0.048</v>
       </c>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
@@ -3045,41 +2985,41 @@
       <c r="O47" s="7"/>
       <c r="P47" s="7"/>
     </row>
-    <row r="48" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B48" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>435151014845</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="H48" s="8" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="I48" s="8" t="n">
+      <c r="G48" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="I48" s="9" t="n">
         <f aca="false">B48*H48</f>
-        <v>0.17</v>
-      </c>
-      <c r="J48" s="8" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="K48" s="8" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J48" s="9" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="K48" s="9" t="n">
         <f aca="false">B48*J48</f>
-        <v>0.048</v>
+        <v>0.726</v>
       </c>
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
@@ -3087,41 +3027,41 @@
       <c r="O48" s="7"/>
       <c r="P48" s="7"/>
     </row>
-    <row r="49" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B49" s="7" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>435151014845</v>
+        <v>5010</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G49" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="H49" s="8" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="I49" s="8" t="n">
+      <c r="G49" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I49" s="9" t="n">
         <f aca="false">B49*H49</f>
-        <v>1.08</v>
-      </c>
-      <c r="J49" s="8" t="n">
-        <v>0.363</v>
-      </c>
-      <c r="K49" s="8" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="J49" s="9" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="K49" s="9" t="n">
         <f aca="false">B49*J49</f>
-        <v>0.726</v>
+        <v>4.324</v>
       </c>
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
@@ -3129,75 +3069,75 @@
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
     </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="B50" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="D50" s="4" t="s">
+    <row r="50" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="E50" s="4" t="n">
-        <v>5010</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G50" s="4" t="s">
+      <c r="B50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="H50" s="6" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="I50" s="6" t="n">
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I50" s="9" t="n">
         <f aca="false">B50*H50</f>
-        <v>7.59</v>
-      </c>
-      <c r="J50" s="6" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="K50" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="9" t="n">
         <f aca="false">B50*J50</f>
-        <v>4.324</v>
-      </c>
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
-      <c r="P50" s="4"/>
-    </row>
-    <row r="51" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
+    </row>
+    <row r="51" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>224</v>
       </c>
       <c r="B51" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I51" s="8" t="n">
+      <c r="D51" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="H51" s="9" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="I51" s="9" t="n">
         <f aca="false">B51*H51</f>
-        <v>5</v>
-      </c>
-      <c r="J51" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K51" s="8" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="J51" s="9" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="K51" s="9" t="n">
         <f aca="false">B51*J51</f>
-        <v>1</v>
+        <v>0.333</v>
       </c>
       <c r="L51" s="7"/>
       <c r="M51" s="7"/>
@@ -3205,276 +3145,258 @@
       <c r="O51" s="7"/>
       <c r="P51" s="7"/>
     </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="B52" s="4" t="n">
+    <row r="52" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="B52" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C52" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E52" s="22" t="s">
-        <v>228</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G52" s="22" t="s">
+      <c r="C52" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="H52" s="6" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="I52" s="6" t="n">
+      <c r="D52" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I52" s="9" t="n">
         <f aca="false">B52*H52</f>
-        <v>0.23</v>
-      </c>
-      <c r="J52" s="6" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="K52" s="6" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J52" s="9"/>
+      <c r="K52" s="9" t="n">
         <f aca="false">B52*J52</f>
-        <v>0.111</v>
-      </c>
-      <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
-      <c r="P52" s="4"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="B53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="7"/>
+      <c r="M52" s="7"/>
+      <c r="N52" s="7"/>
+      <c r="O52" s="7"/>
+      <c r="P52" s="7"/>
+    </row>
+    <row r="53" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B53" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="D53" s="4" t="s">
+      <c r="C53" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D53" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E53" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="H53" s="6" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="I53" s="6" t="n">
+      <c r="E53" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="H53" s="9" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="I53" s="9" t="n">
         <f aca="false">B53*H53</f>
-        <v>0.76</v>
-      </c>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J53" s="9"/>
+      <c r="K53" s="9" t="n">
         <f aca="false">B53*J53</f>
         <v>0</v>
       </c>
-      <c r="L53" s="4"/>
-      <c r="M53" s="4"/>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4"/>
-      <c r="P53" s="4"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="B54" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="D54" s="4" t="s">
+      <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="7"/>
+      <c r="P53" s="7"/>
+    </row>
+    <row r="54" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D54" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E54" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="I54" s="6" t="n">
+      <c r="E54" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="I54" s="9" t="n">
         <f aca="false">B54*H54</f>
-        <v>1.06</v>
-      </c>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="J54" s="9"/>
+      <c r="K54" s="9" t="n">
         <f aca="false">B54*J54</f>
         <v>0</v>
       </c>
-      <c r="L54" s="4"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
-      <c r="P54" s="4"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="B55" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E55" s="4" t="s">
+      <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
+      <c r="O54" s="7"/>
+      <c r="P54" s="7"/>
+    </row>
+    <row r="55" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="F55" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G55" s="4" t="s">
+      <c r="B55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="H55" s="6" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="I55" s="6" t="n">
+      <c r="D55" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G55" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="H55" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I55" s="9" t="n">
         <f aca="false">B55*H55</f>
-        <v>4.14</v>
-      </c>
-      <c r="J55" s="6"/>
-      <c r="K55" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J55" s="9"/>
+      <c r="K55" s="9" t="n">
         <f aca="false">B55*J55</f>
         <v>0</v>
       </c>
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
-      <c r="P55" s="4"/>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="B56" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="D56" s="4" t="s">
+      <c r="L55" s="7"/>
+      <c r="M55" s="7"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="7"/>
+      <c r="P55" s="7"/>
+    </row>
+    <row r="56" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="D56" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E56" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G56" s="22" t="s">
-        <v>245</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I56" s="6" t="n">
+      <c r="E56" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G56" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I56" s="9" t="n">
         <f aca="false">B56*H56</f>
-        <v>0.1</v>
-      </c>
-      <c r="J56" s="6"/>
-      <c r="K56" s="6" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J56" s="9"/>
+      <c r="K56" s="9" t="n">
         <f aca="false">B56*J56</f>
         <v>0</v>
       </c>
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
-      <c r="P56" s="4"/>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="B57" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E57" s="4" t="s">
+      <c r="L56" s="7"/>
+      <c r="M56" s="7"/>
+      <c r="N56" s="7"/>
+      <c r="O56" s="7"/>
+      <c r="P56" s="7"/>
+    </row>
+    <row r="57" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="F57" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G57" s="22" t="s">
+      <c r="B57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="H57" s="6" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I57" s="6" t="n">
+      <c r="D57" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G57" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="H57" s="9" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="I57" s="9" t="n">
         <f aca="false">B57*H57</f>
-        <v>0.52</v>
-      </c>
-      <c r="J57" s="6"/>
-      <c r="K57" s="6" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="J57" s="9"/>
+      <c r="K57" s="9" t="n">
         <f aca="false">B57*J57</f>
         <v>0</v>
       </c>
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
-      <c r="P57" s="4"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="7"/>
+      <c r="P57" s="7"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="B58" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E58" s="22" t="s">
-        <v>252</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G58" s="22" t="s">
-        <v>253</v>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>10.63</v>
-      </c>
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="6"/>
       <c r="I58" s="6" t="n">
         <f aca="false">B58*H58</f>
-        <v>10.63</v>
+        <v>0</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="6" t="n">
@@ -3510,30 +3432,6 @@
       <c r="N59" s="4"/>
       <c r="O59" s="4"/>
       <c r="P59" s="4"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="6"/>
-      <c r="I60" s="6" t="n">
-        <f aca="false">B60*H60</f>
-        <v>0</v>
-      </c>
-      <c r="J60" s="6"/>
-      <c r="K60" s="6" t="n">
-        <f aca="false">B60*J60</f>
-        <v>0</v>
-      </c>
-      <c r="L60" s="4"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="4"/>
-      <c r="O60" s="4"/>
-      <c r="P60" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
New content from latest stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
@@ -809,24 +809,12 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00A933"/>
-        <bgColor rgb="FF008000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -870,7 +858,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -899,31 +887,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -936,66 +912,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF00A933"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -1213,7 +1129,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>21</v>
       </c>
@@ -1232,20 +1148,20 @@
       <c r="F6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="8" t="n">
         <v>0.22</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="8" t="n">
         <f aca="false">B6*H6</f>
         <v>0.88</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="8" t="n">
         <v>0.068</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="8" t="n">
         <f aca="false">B6*J6</f>
         <v>0.272</v>
       </c>
@@ -1255,7 +1171,7 @@
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
     </row>
-    <row r="7" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
@@ -1274,20 +1190,20 @@
       <c r="F7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="8" t="n">
         <f aca="false">B7*H7</f>
         <v>1.1</v>
       </c>
-      <c r="J7" s="9" t="n">
+      <c r="J7" s="8" t="n">
         <v>0.012</v>
       </c>
-      <c r="K7" s="9" t="n">
+      <c r="K7" s="8" t="n">
         <f aca="false">B7*J7</f>
         <v>0.132</v>
       </c>
@@ -1297,7 +1213,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
     </row>
-    <row r="8" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
         <v>32</v>
       </c>
@@ -1316,20 +1232,20 @@
       <c r="F8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="8" t="n">
         <v>0.6</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="8" t="n">
         <f aca="false">B8*H8</f>
         <v>2.4</v>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="J8" s="8" t="n">
         <v>0.187</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K8" s="8" t="n">
         <f aca="false">B8*J8</f>
         <v>0.748</v>
       </c>
@@ -1339,7 +1255,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
     </row>
-    <row r="9" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>37</v>
       </c>
@@ -1358,20 +1274,20 @@
       <c r="F9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="H9" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="I9" s="8" t="n">
         <f aca="false">B9*H9</f>
         <v>0.5</v>
       </c>
-      <c r="J9" s="9" t="n">
+      <c r="J9" s="8" t="n">
         <v>0.023</v>
       </c>
-      <c r="K9" s="9" t="n">
+      <c r="K9" s="8" t="n">
         <f aca="false">B9*J9</f>
         <v>0.115</v>
       </c>
@@ -1381,7 +1297,7 @@
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
     </row>
-    <row r="10" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>42</v>
       </c>
@@ -1400,20 +1316,20 @@
       <c r="F10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="H10" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I10" s="8" t="n">
         <f aca="false">B10*H10</f>
         <v>0.2</v>
       </c>
-      <c r="J10" s="9" t="n">
+      <c r="J10" s="8" t="n">
         <v>0.043</v>
       </c>
-      <c r="K10" s="9" t="n">
+      <c r="K10" s="8" t="n">
         <f aca="false">B10*J10</f>
         <v>0.086</v>
       </c>
@@ -1423,7 +1339,7 @@
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
     </row>
-    <row r="11" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>46</v>
       </c>
@@ -1442,20 +1358,20 @@
       <c r="F11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="8" t="n">
         <v>1.49</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I11" s="8" t="n">
         <f aca="false">B11*H11</f>
         <v>1.49</v>
       </c>
-      <c r="J11" s="9" t="n">
+      <c r="J11" s="8" t="n">
         <v>0.472</v>
       </c>
-      <c r="K11" s="9" t="n">
+      <c r="K11" s="8" t="n">
         <f aca="false">B11*J11</f>
         <v>0.472</v>
       </c>
@@ -1465,7 +1381,7 @@
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
     </row>
-    <row r="12" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>51</v>
       </c>
@@ -1484,20 +1400,20 @@
       <c r="F12" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I12" s="9" t="n">
+      <c r="I12" s="8" t="n">
         <f aca="false">B12*H12</f>
         <v>0.1</v>
       </c>
-      <c r="J12" s="9" t="n">
+      <c r="J12" s="8" t="n">
         <v>0.019</v>
       </c>
-      <c r="K12" s="9" t="n">
+      <c r="K12" s="8" t="n">
         <f aca="false">B12*J12</f>
         <v>0.019</v>
       </c>
@@ -1507,7 +1423,7 @@
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
     </row>
-    <row r="13" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>55</v>
       </c>
@@ -1526,20 +1442,20 @@
       <c r="F13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="H13" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="I13" s="9" t="n">
+      <c r="I13" s="8" t="n">
         <f aca="false">B13*H13</f>
         <v>0.15</v>
       </c>
-      <c r="J13" s="9" t="n">
+      <c r="J13" s="8" t="n">
         <v>0.035</v>
       </c>
-      <c r="K13" s="9" t="n">
+      <c r="K13" s="8" t="n">
         <f aca="false">B13*J13</f>
         <v>0.035</v>
       </c>
@@ -1549,7 +1465,7 @@
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
-    <row r="14" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>60</v>
       </c>
@@ -1568,20 +1484,20 @@
       <c r="F14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I14" s="8" t="n">
         <f aca="false">B14*H14</f>
         <v>0.33</v>
       </c>
-      <c r="J14" s="9" t="n">
+      <c r="J14" s="8" t="n">
         <v>0.128</v>
       </c>
-      <c r="K14" s="9" t="n">
+      <c r="K14" s="8" t="n">
         <f aca="false">B14*J14</f>
         <v>0.128</v>
       </c>
@@ -1591,7 +1507,7 @@
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
     </row>
-    <row r="15" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
         <v>65</v>
       </c>
@@ -1610,20 +1526,20 @@
       <c r="F15" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="8" t="n">
         <v>0.48</v>
       </c>
-      <c r="I15" s="9" t="n">
+      <c r="I15" s="8" t="n">
         <f aca="false">B15*H15</f>
         <v>0.48</v>
       </c>
-      <c r="J15" s="9" t="n">
+      <c r="J15" s="8" t="n">
         <v>0.189</v>
       </c>
-      <c r="K15" s="9" t="n">
+      <c r="K15" s="8" t="n">
         <f aca="false">B15*J15</f>
         <v>0.189</v>
       </c>
@@ -1633,7 +1549,7 @@
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
     </row>
-    <row r="16" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>69</v>
       </c>
@@ -1652,20 +1568,20 @@
       <c r="F16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="H16" s="9" t="n">
+      <c r="H16" s="8" t="n">
         <v>0.62</v>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="I16" s="8" t="n">
         <f aca="false">B16*H16</f>
         <v>1.86</v>
       </c>
-      <c r="J16" s="9" t="n">
+      <c r="J16" s="8" t="n">
         <v>0.246</v>
       </c>
-      <c r="K16" s="9" t="n">
+      <c r="K16" s="8" t="n">
         <f aca="false">B16*J16</f>
         <v>0.738</v>
       </c>
@@ -1675,7 +1591,7 @@
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
     </row>
-    <row r="17" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>73</v>
       </c>
@@ -1694,20 +1610,20 @@
       <c r="F17" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="9" t="n">
+      <c r="H17" s="8" t="n">
         <v>0.78</v>
       </c>
-      <c r="I17" s="9" t="n">
+      <c r="I17" s="8" t="n">
         <f aca="false">B17*H17</f>
         <v>0.78</v>
       </c>
-      <c r="J17" s="9" t="n">
+      <c r="J17" s="8" t="n">
         <v>0.484</v>
       </c>
-      <c r="K17" s="9" t="n">
+      <c r="K17" s="8" t="n">
         <f aca="false">B17*J17</f>
         <v>0.484</v>
       </c>
@@ -1717,7 +1633,7 @@
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
     </row>
-    <row r="18" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>78</v>
       </c>
@@ -1736,20 +1652,20 @@
       <c r="F18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="9" t="n">
+      <c r="H18" s="8" t="n">
         <v>0.79</v>
       </c>
-      <c r="I18" s="9" t="n">
+      <c r="I18" s="8" t="n">
         <f aca="false">B18*H18</f>
         <v>0.79</v>
       </c>
-      <c r="J18" s="9" t="n">
+      <c r="J18" s="8" t="n">
         <v>0.369</v>
       </c>
-      <c r="K18" s="9" t="n">
+      <c r="K18" s="8" t="n">
         <f aca="false">B18*J18</f>
         <v>0.369</v>
       </c>
@@ -1759,7 +1675,7 @@
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
     </row>
-    <row r="19" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>83</v>
       </c>
@@ -1778,20 +1694,20 @@
       <c r="F19" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="9" t="n">
+      <c r="H19" s="8" t="n">
         <v>0.27</v>
       </c>
-      <c r="I19" s="9" t="n">
+      <c r="I19" s="8" t="n">
         <f aca="false">B19*H19</f>
         <v>0.54</v>
       </c>
-      <c r="J19" s="9" t="n">
+      <c r="J19" s="8" t="n">
         <v>0.049</v>
       </c>
-      <c r="K19" s="9" t="n">
+      <c r="K19" s="8" t="n">
         <f aca="false">B19*J19</f>
         <v>0.098</v>
       </c>
@@ -1801,7 +1717,7 @@
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
     </row>
-    <row r="20" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>88</v>
       </c>
@@ -1820,20 +1736,20 @@
       <c r="F20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="8" t="n">
         <v>0.36</v>
       </c>
-      <c r="I20" s="9" t="n">
+      <c r="I20" s="8" t="n">
         <f aca="false">B20*H20</f>
         <v>0.36</v>
       </c>
-      <c r="J20" s="9" t="n">
+      <c r="J20" s="8" t="n">
         <v>0.076</v>
       </c>
-      <c r="K20" s="9" t="n">
+      <c r="K20" s="8" t="n">
         <f aca="false">B20*J20</f>
         <v>0.076</v>
       </c>
@@ -1843,7 +1759,7 @@
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
     </row>
-    <row r="21" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>93</v>
       </c>
@@ -1862,20 +1778,20 @@
       <c r="F21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="H21" s="9" t="n">
+      <c r="H21" s="8" t="n">
         <v>1.11</v>
       </c>
-      <c r="I21" s="9" t="n">
+      <c r="I21" s="8" t="n">
         <f aca="false">B21*H21</f>
         <v>5.55</v>
       </c>
-      <c r="J21" s="9" t="n">
+      <c r="J21" s="8" t="n">
         <v>0.343</v>
       </c>
-      <c r="K21" s="9" t="n">
+      <c r="K21" s="8" t="n">
         <f aca="false">B21*J21</f>
         <v>1.715</v>
       </c>
@@ -1885,7 +1801,7 @@
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
     </row>
-    <row r="22" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>98</v>
       </c>
@@ -1904,20 +1820,20 @@
       <c r="F22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="9" t="n">
+      <c r="H22" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="I22" s="9" t="n">
+      <c r="I22" s="8" t="n">
         <f aca="false">B22*H22</f>
         <v>0.15</v>
       </c>
-      <c r="J22" s="9" t="n">
+      <c r="J22" s="8" t="n">
         <v>0.045</v>
       </c>
-      <c r="K22" s="9" t="n">
+      <c r="K22" s="8" t="n">
         <f aca="false">B22*J22</f>
         <v>0.045</v>
       </c>
@@ -1927,7 +1843,7 @@
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
     </row>
-    <row r="23" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>102</v>
       </c>
@@ -1946,20 +1862,20 @@
       <c r="F23" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="H23" s="9" t="n">
+      <c r="H23" s="8" t="n">
         <v>0.71</v>
       </c>
-      <c r="I23" s="9" t="n">
+      <c r="I23" s="8" t="n">
         <f aca="false">B23*H23</f>
         <v>0.71</v>
       </c>
-      <c r="J23" s="9" t="n">
+      <c r="J23" s="8" t="n">
         <v>0.342</v>
       </c>
-      <c r="K23" s="9" t="n">
+      <c r="K23" s="8" t="n">
         <f aca="false">B23*J23</f>
         <v>0.342</v>
       </c>
@@ -1969,7 +1885,7 @@
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
     </row>
-    <row r="24" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
         <v>107</v>
       </c>
@@ -1988,20 +1904,20 @@
       <c r="F24" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="H24" s="9" t="n">
+      <c r="H24" s="8" t="n">
         <v>0.71</v>
       </c>
-      <c r="I24" s="9" t="n">
+      <c r="I24" s="8" t="n">
         <f aca="false">B24*H24</f>
         <v>0.71</v>
       </c>
-      <c r="J24" s="9" t="n">
+      <c r="J24" s="8" t="n">
         <v>0.342</v>
       </c>
-      <c r="K24" s="9" t="n">
+      <c r="K24" s="8" t="n">
         <f aca="false">B24*J24</f>
         <v>0.342</v>
       </c>
@@ -2011,7 +1927,7 @@
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
     </row>
-    <row r="25" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
         <v>111</v>
       </c>
@@ -2030,20 +1946,20 @@
       <c r="F25" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H25" s="9" t="n">
+      <c r="H25" s="8" t="n">
         <v>6.71</v>
       </c>
-      <c r="I25" s="9" t="n">
+      <c r="I25" s="8" t="n">
         <f aca="false">B25*H25</f>
         <v>6.71</v>
       </c>
-      <c r="J25" s="9" t="n">
+      <c r="J25" s="8" t="n">
         <v>3.98</v>
       </c>
-      <c r="K25" s="9" t="n">
+      <c r="K25" s="8" t="n">
         <f aca="false">B25*J25</f>
         <v>3.98</v>
       </c>
@@ -2053,7 +1969,7 @@
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
     </row>
-    <row r="26" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
         <v>115</v>
       </c>
@@ -2072,20 +1988,20 @@
       <c r="F26" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="H26" s="9" t="n">
+      <c r="H26" s="8" t="n">
         <v>0.81</v>
       </c>
-      <c r="I26" s="9" t="n">
+      <c r="I26" s="8" t="n">
         <f aca="false">B26*H26</f>
         <v>0.81</v>
       </c>
-      <c r="J26" s="9" t="n">
+      <c r="J26" s="8" t="n">
         <v>0.38</v>
       </c>
-      <c r="K26" s="9" t="n">
+      <c r="K26" s="8" t="n">
         <f aca="false">B26*J26</f>
         <v>0.38</v>
       </c>
@@ -2103,7 +2019,7 @@
       </c>
       <c r="P26" s="7"/>
     </row>
-    <row r="27" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
         <v>122</v>
       </c>
@@ -2122,20 +2038,20 @@
       <c r="F27" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="H27" s="9" t="n">
+      <c r="H27" s="8" t="n">
         <v>3.55</v>
       </c>
-      <c r="I27" s="9" t="n">
+      <c r="I27" s="8" t="n">
         <f aca="false">B27*H27</f>
         <v>3.55</v>
       </c>
-      <c r="J27" s="9" t="n">
+      <c r="J27" s="8" t="n">
         <v>1.31</v>
       </c>
-      <c r="K27" s="9" t="n">
+      <c r="K27" s="8" t="n">
         <f aca="false">B27*J27</f>
         <v>1.31</v>
       </c>
@@ -2145,7 +2061,7 @@
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
     </row>
-    <row r="28" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
         <v>127</v>
       </c>
@@ -2164,20 +2080,20 @@
       <c r="F28" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G28" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="H28" s="9" t="n">
+      <c r="H28" s="8" t="n">
         <v>4.03</v>
       </c>
-      <c r="I28" s="9" t="n">
+      <c r="I28" s="8" t="n">
         <f aca="false">B28*H28</f>
         <v>4.03</v>
       </c>
-      <c r="J28" s="9" t="n">
+      <c r="J28" s="8" t="n">
         <v>2.4</v>
       </c>
-      <c r="K28" s="9" t="n">
+      <c r="K28" s="8" t="n">
         <f aca="false">B28*J28</f>
         <v>2.4</v>
       </c>
@@ -2187,7 +2103,7 @@
       <c r="O28" s="7"/>
       <c r="P28" s="7"/>
     </row>
-    <row r="29" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>132</v>
       </c>
@@ -2206,20 +2122,20 @@
       <c r="F29" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="9" t="n">
+      <c r="H29" s="8" t="n">
         <v>1.89</v>
       </c>
-      <c r="I29" s="9" t="n">
+      <c r="I29" s="8" t="n">
         <f aca="false">B29*H29</f>
         <v>1.89</v>
       </c>
-      <c r="J29" s="9" t="n">
+      <c r="J29" s="8" t="n">
         <v>1.22</v>
       </c>
-      <c r="K29" s="9" t="n">
+      <c r="K29" s="8" t="n">
         <f aca="false">B29*J29</f>
         <v>1.22</v>
       </c>
@@ -2229,7 +2145,7 @@
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
     </row>
-    <row r="30" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
         <v>137</v>
       </c>
@@ -2248,20 +2164,20 @@
       <c r="F30" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="H30" s="9" t="n">
+      <c r="H30" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I30" s="9" t="n">
+      <c r="I30" s="8" t="n">
         <f aca="false">B30*H30</f>
         <v>0.3</v>
       </c>
-      <c r="J30" s="9" t="n">
+      <c r="J30" s="8" t="n">
         <v>0.071</v>
       </c>
-      <c r="K30" s="9" t="n">
+      <c r="K30" s="8" t="n">
         <f aca="false">B30*J30</f>
         <v>0.213</v>
       </c>
@@ -2271,7 +2187,7 @@
       <c r="O30" s="7"/>
       <c r="P30" s="7"/>
     </row>
-    <row r="31" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>142</v>
       </c>
@@ -2290,20 +2206,20 @@
       <c r="F31" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="9" t="n">
+      <c r="H31" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I31" s="9" t="n">
+      <c r="I31" s="8" t="n">
         <f aca="false">B31*H31</f>
         <v>0.17</v>
       </c>
-      <c r="J31" s="9" t="n">
+      <c r="J31" s="8" t="n">
         <v>0.163</v>
       </c>
-      <c r="K31" s="9" t="n">
+      <c r="K31" s="8" t="n">
         <f aca="false">B31*J31</f>
         <v>0.163</v>
       </c>
@@ -2313,7 +2229,7 @@
       <c r="O31" s="7"/>
       <c r="P31" s="7"/>
     </row>
-    <row r="32" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
         <v>147</v>
       </c>
@@ -2332,20 +2248,20 @@
       <c r="F32" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="H32" s="9" t="n">
+      <c r="H32" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I32" s="9" t="n">
+      <c r="I32" s="8" t="n">
         <f aca="false">B32*H32</f>
         <v>0.66</v>
       </c>
-      <c r="J32" s="9" t="n">
+      <c r="J32" s="8" t="n">
         <v>0.199</v>
       </c>
-      <c r="K32" s="9" t="n">
+      <c r="K32" s="8" t="n">
         <f aca="false">B32*J32</f>
         <v>0.398</v>
       </c>
@@ -2355,7 +2271,7 @@
       <c r="O32" s="7"/>
       <c r="P32" s="7"/>
     </row>
-    <row r="33" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
         <v>151</v>
       </c>
@@ -2374,20 +2290,20 @@
       <c r="F33" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="H33" s="9" t="n">
+      <c r="H33" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="I33" s="9" t="n">
+      <c r="I33" s="8" t="n">
         <f aca="false">B33*H33</f>
         <v>4.56</v>
       </c>
-      <c r="J33" s="9" t="n">
+      <c r="J33" s="8" t="n">
         <v>0.303</v>
       </c>
-      <c r="K33" s="9" t="n">
+      <c r="K33" s="8" t="n">
         <f aca="false">B33*J33</f>
         <v>1.818</v>
       </c>
@@ -2397,7 +2313,7 @@
       <c r="O33" s="7"/>
       <c r="P33" s="7"/>
     </row>
-    <row r="34" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
         <v>156</v>
       </c>
@@ -2416,20 +2332,20 @@
       <c r="F34" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G34" s="8" t="s">
+      <c r="G34" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="H34" s="9" t="n">
+      <c r="H34" s="8" t="n">
         <v>0.14</v>
       </c>
-      <c r="I34" s="9" t="n">
+      <c r="I34" s="8" t="n">
         <f aca="false">B34*H34</f>
         <v>0.14</v>
       </c>
-      <c r="J34" s="9" t="n">
+      <c r="J34" s="8" t="n">
         <v>0.42</v>
       </c>
-      <c r="K34" s="9" t="n">
+      <c r="K34" s="8" t="n">
         <f aca="false">B34*J34</f>
         <v>0.42</v>
       </c>
@@ -2439,7 +2355,7 @@
       <c r="O34" s="7"/>
       <c r="P34" s="7"/>
     </row>
-    <row r="35" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
         <v>161</v>
       </c>
@@ -2458,20 +2374,20 @@
       <c r="F35" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G35" s="8" t="s">
+      <c r="G35" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="H35" s="9" t="n">
+      <c r="H35" s="8" t="n">
         <v>0.19</v>
       </c>
-      <c r="I35" s="9" t="n">
+      <c r="I35" s="8" t="n">
         <f aca="false">B35*H35</f>
         <v>0.38</v>
       </c>
-      <c r="J35" s="9" t="n">
+      <c r="J35" s="8" t="n">
         <v>0.015</v>
       </c>
-      <c r="K35" s="9" t="n">
+      <c r="K35" s="8" t="n">
         <f aca="false">B35*J35</f>
         <v>0.03</v>
       </c>
@@ -2481,7 +2397,7 @@
       <c r="O35" s="7"/>
       <c r="P35" s="7"/>
     </row>
-    <row r="36" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>165</v>
       </c>
@@ -2500,20 +2416,20 @@
       <c r="F36" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G36" s="8" t="s">
+      <c r="G36" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="H36" s="9" t="n">
+      <c r="H36" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I36" s="9" t="n">
+      <c r="I36" s="8" t="n">
         <f aca="false">B36*H36</f>
         <v>0.1</v>
       </c>
-      <c r="J36" s="9" t="n">
+      <c r="J36" s="8" t="n">
         <v>0.021</v>
       </c>
-      <c r="K36" s="9" t="n">
+      <c r="K36" s="8" t="n">
         <f aca="false">B36*J36</f>
         <v>0.021</v>
       </c>
@@ -2523,7 +2439,7 @@
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
     </row>
-    <row r="37" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>169</v>
       </c>
@@ -2542,20 +2458,20 @@
       <c r="F37" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="H37" s="9" t="n">
+      <c r="H37" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I37" s="9" t="n">
+      <c r="I37" s="8" t="n">
         <f aca="false">B37*H37</f>
         <v>0.1</v>
       </c>
-      <c r="J37" s="9" t="n">
+      <c r="J37" s="8" t="n">
         <v>0.043</v>
       </c>
-      <c r="K37" s="9" t="n">
+      <c r="K37" s="8" t="n">
         <f aca="false">B37*J37</f>
         <v>0.043</v>
       </c>
@@ -2565,7 +2481,7 @@
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
     </row>
-    <row r="38" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>174</v>
       </c>
@@ -2584,20 +2500,20 @@
       <c r="F38" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G38" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="H38" s="9" t="n">
+      <c r="H38" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I38" s="9" t="n">
+      <c r="I38" s="8" t="n">
         <f aca="false">B38*H38</f>
         <v>1.32</v>
       </c>
-      <c r="J38" s="9" t="n">
+      <c r="J38" s="8" t="n">
         <v>0.031</v>
       </c>
-      <c r="K38" s="9" t="n">
+      <c r="K38" s="8" t="n">
         <f aca="false">B38*J38</f>
         <v>0.372</v>
       </c>
@@ -2607,7 +2523,7 @@
       <c r="O38" s="7"/>
       <c r="P38" s="7"/>
     </row>
-    <row r="39" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>178</v>
       </c>
@@ -2626,20 +2542,20 @@
       <c r="F39" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G39" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="9" t="n">
+      <c r="H39" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I39" s="9" t="n">
+      <c r="I39" s="8" t="n">
         <f aca="false">B39*H39</f>
         <v>0.1</v>
       </c>
-      <c r="J39" s="9" t="n">
+      <c r="J39" s="8" t="n">
         <v>0.013</v>
       </c>
-      <c r="K39" s="9" t="n">
+      <c r="K39" s="8" t="n">
         <f aca="false">B39*J39</f>
         <v>0.013</v>
       </c>
@@ -2649,7 +2565,7 @@
       <c r="O39" s="7"/>
       <c r="P39" s="7"/>
     </row>
-    <row r="40" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>182</v>
       </c>
@@ -2668,20 +2584,20 @@
       <c r="F40" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="G40" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="H40" s="9" t="n">
+      <c r="H40" s="8" t="n">
         <v>0.12</v>
       </c>
-      <c r="I40" s="9" t="n">
+      <c r="I40" s="8" t="n">
         <f aca="false">B40*H40</f>
         <v>0.72</v>
       </c>
-      <c r="J40" s="9" t="n">
+      <c r="J40" s="8" t="n">
         <v>0.041</v>
       </c>
-      <c r="K40" s="9" t="n">
+      <c r="K40" s="8" t="n">
         <f aca="false">B40*J40</f>
         <v>0.246</v>
       </c>
@@ -2691,7 +2607,7 @@
       <c r="O40" s="7"/>
       <c r="P40" s="7"/>
     </row>
-    <row r="41" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
         <v>186</v>
       </c>
@@ -2710,20 +2626,20 @@
       <c r="F41" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="H41" s="9" t="n">
+      <c r="H41" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I41" s="9" t="n">
+      <c r="I41" s="8" t="n">
         <f aca="false">B41*H41</f>
         <v>0.11</v>
       </c>
-      <c r="J41" s="9" t="n">
+      <c r="J41" s="8" t="n">
         <v>0.009</v>
       </c>
-      <c r="K41" s="9" t="n">
+      <c r="K41" s="8" t="n">
         <f aca="false">B41*J41</f>
         <v>0.009</v>
       </c>
@@ -2733,7 +2649,7 @@
       <c r="O41" s="7"/>
       <c r="P41" s="7"/>
     </row>
-    <row r="42" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
         <v>190</v>
       </c>
@@ -2752,20 +2668,20 @@
       <c r="F42" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G42" s="8" t="s">
+      <c r="G42" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H42" s="9" t="n">
+      <c r="H42" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I42" s="9" t="n">
+      <c r="I42" s="8" t="n">
         <f aca="false">B42*H42</f>
         <v>0.1</v>
       </c>
-      <c r="J42" s="9" t="n">
+      <c r="J42" s="8" t="n">
         <v>0.042</v>
       </c>
-      <c r="K42" s="9" t="n">
+      <c r="K42" s="8" t="n">
         <f aca="false">B42*J42</f>
         <v>0.042</v>
       </c>
@@ -2775,7 +2691,7 @@
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
     </row>
-    <row r="43" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
         <v>194</v>
       </c>
@@ -2794,20 +2710,20 @@
       <c r="F43" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G43" s="8" t="s">
+      <c r="G43" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="H43" s="9" t="n">
+      <c r="H43" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I43" s="9" t="n">
+      <c r="I43" s="8" t="n">
         <f aca="false">B43*H43</f>
         <v>0.22</v>
       </c>
-      <c r="J43" s="9" t="n">
+      <c r="J43" s="8" t="n">
         <v>0.031</v>
       </c>
-      <c r="K43" s="9" t="n">
+      <c r="K43" s="8" t="n">
         <f aca="false">B43*J43</f>
         <v>0.062</v>
       </c>
@@ -2817,7 +2733,7 @@
       <c r="O43" s="7"/>
       <c r="P43" s="7"/>
     </row>
-    <row r="44" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>198</v>
       </c>
@@ -2836,20 +2752,20 @@
       <c r="F44" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G44" s="8" t="s">
+      <c r="G44" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="H44" s="9" t="n">
+      <c r="H44" s="8" t="n">
         <v>0.24</v>
       </c>
-      <c r="I44" s="9" t="n">
+      <c r="I44" s="8" t="n">
         <f aca="false">B44*H44</f>
         <v>0.24</v>
       </c>
-      <c r="J44" s="9" t="n">
+      <c r="J44" s="8" t="n">
         <v>0.139</v>
       </c>
-      <c r="K44" s="9" t="n">
+      <c r="K44" s="8" t="n">
         <f aca="false">B44*J44</f>
         <v>0.139</v>
       </c>
@@ -2859,7 +2775,7 @@
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
     </row>
-    <row r="45" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
         <v>202</v>
       </c>
@@ -2878,20 +2794,20 @@
       <c r="F45" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G45" s="8" t="s">
+      <c r="G45" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="H45" s="9" t="n">
+      <c r="H45" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I45" s="9" t="n">
+      <c r="I45" s="8" t="n">
         <f aca="false">B45*H45</f>
         <v>0.34</v>
       </c>
-      <c r="J45" s="9" t="n">
+      <c r="J45" s="8" t="n">
         <v>0.051</v>
       </c>
-      <c r="K45" s="9" t="n">
+      <c r="K45" s="8" t="n">
         <f aca="false">B45*J45</f>
         <v>0.102</v>
       </c>
@@ -2901,7 +2817,7 @@
       <c r="O45" s="7"/>
       <c r="P45" s="7"/>
     </row>
-    <row r="46" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
         <v>206</v>
       </c>
@@ -2920,20 +2836,20 @@
       <c r="F46" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G46" s="8" t="s">
+      <c r="G46" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="H46" s="9" t="n">
+      <c r="H46" s="8" t="n">
         <v>0.14</v>
       </c>
-      <c r="I46" s="9" t="n">
+      <c r="I46" s="8" t="n">
         <f aca="false">B46*H46</f>
         <v>0.14</v>
       </c>
-      <c r="J46" s="9" t="n">
+      <c r="J46" s="8" t="n">
         <v>0.052</v>
       </c>
-      <c r="K46" s="9" t="n">
+      <c r="K46" s="8" t="n">
         <f aca="false">B46*J46</f>
         <v>0.052</v>
       </c>
@@ -2943,7 +2859,7 @@
       <c r="O46" s="7"/>
       <c r="P46" s="7"/>
     </row>
-    <row r="47" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>210</v>
       </c>
@@ -2962,20 +2878,20 @@
       <c r="F47" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G47" s="8" t="s">
+      <c r="G47" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="H47" s="9" t="n">
+      <c r="H47" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I47" s="9" t="n">
+      <c r="I47" s="8" t="n">
         <f aca="false">B47*H47</f>
         <v>0.17</v>
       </c>
-      <c r="J47" s="9" t="n">
+      <c r="J47" s="8" t="n">
         <v>0.048</v>
       </c>
-      <c r="K47" s="9" t="n">
+      <c r="K47" s="8" t="n">
         <f aca="false">B47*J47</f>
         <v>0.048</v>
       </c>
@@ -2985,7 +2901,7 @@
       <c r="O47" s="7"/>
       <c r="P47" s="7"/>
     </row>
-    <row r="48" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>214</v>
       </c>
@@ -3004,20 +2920,20 @@
       <c r="F48" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G48" s="8" t="s">
+      <c r="G48" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="H48" s="9" t="n">
+      <c r="H48" s="8" t="n">
         <v>0.54</v>
       </c>
-      <c r="I48" s="9" t="n">
+      <c r="I48" s="8" t="n">
         <f aca="false">B48*H48</f>
         <v>1.08</v>
       </c>
-      <c r="J48" s="9" t="n">
+      <c r="J48" s="8" t="n">
         <v>0.363</v>
       </c>
-      <c r="K48" s="9" t="n">
+      <c r="K48" s="8" t="n">
         <f aca="false">B48*J48</f>
         <v>0.726</v>
       </c>
@@ -3027,7 +2943,7 @@
       <c r="O48" s="7"/>
       <c r="P48" s="7"/>
     </row>
-    <row r="49" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>218</v>
       </c>
@@ -3046,20 +2962,20 @@
       <c r="F49" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G49" s="8" t="s">
+      <c r="G49" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="H49" s="9" t="n">
+      <c r="H49" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I49" s="9" t="n">
+      <c r="I49" s="8" t="n">
         <f aca="false">B49*H49</f>
         <v>7.59</v>
       </c>
-      <c r="J49" s="9" t="n">
+      <c r="J49" s="8" t="n">
         <v>0.188</v>
       </c>
-      <c r="K49" s="9" t="n">
+      <c r="K49" s="8" t="n">
         <f aca="false">B49*J49</f>
         <v>4.324</v>
       </c>
@@ -3069,7 +2985,7 @@
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
     </row>
-    <row r="50" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>222</v>
       </c>
@@ -3083,17 +2999,17 @@
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
       <c r="G50" s="7"/>
-      <c r="H50" s="9" t="n">
+      <c r="H50" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I50" s="9" t="n">
+      <c r="I50" s="8" t="n">
         <f aca="false">B50*H50</f>
         <v>5</v>
       </c>
-      <c r="J50" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K50" s="9" t="n">
+      <c r="J50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="8" t="n">
         <f aca="false">B50*J50</f>
         <v>1</v>
       </c>
@@ -3103,7 +3019,7 @@
       <c r="O50" s="7"/>
       <c r="P50" s="7"/>
     </row>
-    <row r="51" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>224</v>
       </c>
@@ -3116,26 +3032,26 @@
       <c r="D51" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E51" s="12" t="s">
+      <c r="E51" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G51" s="13" t="s">
+      <c r="G51" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="H51" s="9" t="n">
+      <c r="H51" s="8" t="n">
         <v>0.23</v>
       </c>
-      <c r="I51" s="9" t="n">
+      <c r="I51" s="8" t="n">
         <f aca="false">B51*H51</f>
         <v>0.69</v>
       </c>
-      <c r="J51" s="9" t="n">
+      <c r="J51" s="8" t="n">
         <v>0.111</v>
       </c>
-      <c r="K51" s="9" t="n">
+      <c r="K51" s="8" t="n">
         <f aca="false">B51*J51</f>
         <v>0.333</v>
       </c>
@@ -3145,7 +3061,7 @@
       <c r="O51" s="7"/>
       <c r="P51" s="7"/>
     </row>
-    <row r="52" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>228</v>
       </c>
@@ -3164,18 +3080,18 @@
       <c r="F52" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G52" s="8" t="s">
+      <c r="G52" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="H52" s="9" t="n">
+      <c r="H52" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="I52" s="9" t="n">
+      <c r="I52" s="8" t="n">
         <f aca="false">B52*H52</f>
         <v>0.76</v>
       </c>
-      <c r="J52" s="9"/>
-      <c r="K52" s="9" t="n">
+      <c r="J52" s="8"/>
+      <c r="K52" s="8" t="n">
         <f aca="false">B52*J52</f>
         <v>0</v>
       </c>
@@ -3185,7 +3101,7 @@
       <c r="O52" s="7"/>
       <c r="P52" s="7"/>
     </row>
-    <row r="53" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>232</v>
       </c>
@@ -3204,18 +3120,18 @@
       <c r="F53" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G53" s="8" t="s">
+      <c r="G53" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="H53" s="9" t="n">
+      <c r="H53" s="8" t="n">
         <v>1.06</v>
       </c>
-      <c r="I53" s="9" t="n">
+      <c r="I53" s="8" t="n">
         <f aca="false">B53*H53</f>
         <v>1.06</v>
       </c>
-      <c r="J53" s="9"/>
-      <c r="K53" s="9" t="n">
+      <c r="J53" s="8"/>
+      <c r="K53" s="8" t="n">
         <f aca="false">B53*J53</f>
         <v>0</v>
       </c>
@@ -3225,7 +3141,7 @@
       <c r="O53" s="7"/>
       <c r="P53" s="7"/>
     </row>
-    <row r="54" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
         <v>236</v>
       </c>
@@ -3244,18 +3160,18 @@
       <c r="F54" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G54" s="8" t="s">
+      <c r="G54" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="H54" s="9" t="n">
+      <c r="H54" s="8" t="n">
         <v>1.38</v>
       </c>
-      <c r="I54" s="9" t="n">
+      <c r="I54" s="8" t="n">
         <f aca="false">B54*H54</f>
         <v>4.14</v>
       </c>
-      <c r="J54" s="9"/>
-      <c r="K54" s="9" t="n">
+      <c r="J54" s="8"/>
+      <c r="K54" s="8" t="n">
         <f aca="false">B54*J54</f>
         <v>0</v>
       </c>
@@ -3265,7 +3181,7 @@
       <c r="O54" s="7"/>
       <c r="P54" s="7"/>
     </row>
-    <row r="55" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>240</v>
       </c>
@@ -3284,18 +3200,18 @@
       <c r="F55" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G55" s="13" t="s">
+      <c r="G55" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="H55" s="9" t="n">
+      <c r="H55" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I55" s="9" t="n">
+      <c r="I55" s="8" t="n">
         <f aca="false">B55*H55</f>
         <v>0.1</v>
       </c>
-      <c r="J55" s="9"/>
-      <c r="K55" s="9" t="n">
+      <c r="J55" s="8"/>
+      <c r="K55" s="8" t="n">
         <f aca="false">B55*J55</f>
         <v>0</v>
       </c>
@@ -3305,7 +3221,7 @@
       <c r="O55" s="7"/>
       <c r="P55" s="7"/>
     </row>
-    <row r="56" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>244</v>
       </c>
@@ -3324,18 +3240,18 @@
       <c r="F56" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G56" s="13" t="s">
+      <c r="G56" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="H56" s="9" t="n">
+      <c r="H56" s="8" t="n">
         <v>0.13</v>
       </c>
-      <c r="I56" s="9" t="n">
+      <c r="I56" s="8" t="n">
         <f aca="false">B56*H56</f>
         <v>0.52</v>
       </c>
-      <c r="J56" s="9"/>
-      <c r="K56" s="9" t="n">
+      <c r="J56" s="8"/>
+      <c r="K56" s="8" t="n">
         <f aca="false">B56*J56</f>
         <v>0</v>
       </c>
@@ -3345,7 +3261,7 @@
       <c r="O56" s="7"/>
       <c r="P56" s="7"/>
     </row>
-    <row r="57" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>248</v>
       </c>
@@ -3358,24 +3274,24 @@
       <c r="D57" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E57" s="12" t="s">
+      <c r="E57" s="10" t="s">
         <v>250</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G57" s="13" t="s">
+      <c r="G57" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="H57" s="9" t="n">
+      <c r="H57" s="8" t="n">
         <v>10.63</v>
       </c>
-      <c r="I57" s="9" t="n">
+      <c r="I57" s="8" t="n">
         <f aca="false">B57*H57</f>
         <v>10.63</v>
       </c>
-      <c r="J57" s="9"/>
-      <c r="K57" s="9" t="n">
+      <c r="J57" s="8"/>
+      <c r="K57" s="8" t="n">
         <f aca="false">B57*J57</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added new files from stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-01/P1012202501-BOM V1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="261">
   <si>
     <t xml:space="preserve">Project:</t>
   </si>
@@ -776,6 +776,33 @@
   </si>
   <si>
     <t xml:space="preserve">490-CFM-4010-03-22 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heat Sink for IC6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HS8.8x8.5x8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSB01-080808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2223-HSB01-080808-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tape for Heatsink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSTAPE8x8x0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TG-T1000-8-8-0.25-5PT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1168-TG-T1000-8-8-0.25-5PT-ND</t>
   </si>
 </sst>
 </file>
@@ -809,12 +836,18 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF729FCF"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -858,7 +891,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -883,19 +916,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -912,6 +941,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF729FCF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1032,19 +1121,19 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.77"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="4" min="4" style="1" width="20.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="31.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="16.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="21.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="16.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.52"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="31.76"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="2" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="9" min="9" style="2" width="20.77"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="2" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="2" width="21.04"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="13" min="13" style="1" width="14.52"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="14" min="14" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="15" min="15" style="1" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="16" min="16" style="1" width="14.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1060,7 +1149,7 @@
       </c>
       <c r="I1" s="2" t="n">
         <f aca="false">SUM(I6:I61)</f>
-        <v>77.51</v>
+        <v>78.49</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>3</v>
@@ -1080,75 +1169,75 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="L5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="4" t="s">
+      <c r="P5" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>26</v>
       </c>
       <c r="H6" s="8" t="n">
@@ -1165,32 +1254,32 @@
         <f aca="false">B6*J6</f>
         <v>0.272</v>
       </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-    </row>
-    <row r="7" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+    </row>
+    <row r="7" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="F7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>31</v>
       </c>
       <c r="H7" s="8" t="n">
@@ -1207,32 +1296,32 @@
         <f aca="false">B7*J7</f>
         <v>0.132</v>
       </c>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-    </row>
-    <row r="8" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+    </row>
+    <row r="8" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="F8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H8" s="8" t="n">
@@ -1249,32 +1338,32 @@
         <f aca="false">B8*J8</f>
         <v>0.748</v>
       </c>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-    </row>
-    <row r="9" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+    </row>
+    <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="7" t="s">
+      <c r="F9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>41</v>
       </c>
       <c r="H9" s="8" t="n">
@@ -1291,32 +1380,32 @@
         <f aca="false">B9*J9</f>
         <v>0.115</v>
       </c>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-    </row>
-    <row r="10" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+    </row>
+    <row r="10" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="F10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>45</v>
       </c>
       <c r="H10" s="8" t="n">
@@ -1333,32 +1422,32 @@
         <f aca="false">B10*J10</f>
         <v>0.086</v>
       </c>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-    </row>
-    <row r="11" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+    </row>
+    <row r="11" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="7" t="s">
+      <c r="F11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H11" s="8" t="n">
@@ -1375,32 +1464,32 @@
         <f aca="false">B11*J11</f>
         <v>0.472</v>
       </c>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-    </row>
-    <row r="12" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+    </row>
+    <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="7" t="s">
+      <c r="F12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="8" t="n">
@@ -1417,32 +1506,32 @@
         <f aca="false">B12*J12</f>
         <v>0.019</v>
       </c>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-    </row>
-    <row r="13" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+    </row>
+    <row r="13" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="7" t="s">
+      <c r="F13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>59</v>
       </c>
       <c r="H13" s="8" t="n">
@@ -1459,32 +1548,32 @@
         <f aca="false">B13*J13</f>
         <v>0.035</v>
       </c>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-    </row>
-    <row r="14" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+    </row>
+    <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="B14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="7" t="s">
+      <c r="F14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>64</v>
       </c>
       <c r="H14" s="8" t="n">
@@ -1501,32 +1590,32 @@
         <f aca="false">B14*J14</f>
         <v>0.128</v>
       </c>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-    </row>
-    <row r="15" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+    </row>
+    <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="B15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="7" t="s">
+      <c r="F15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>68</v>
       </c>
       <c r="H15" s="8" t="n">
@@ -1543,32 +1632,32 @@
         <f aca="false">B15*J15</f>
         <v>0.189</v>
       </c>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-    </row>
-    <row r="16" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+    </row>
+    <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="7" t="s">
+      <c r="F16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>72</v>
       </c>
       <c r="H16" s="8" t="n">
@@ -1585,32 +1674,32 @@
         <f aca="false">B16*J16</f>
         <v>0.738</v>
       </c>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-    </row>
-    <row r="17" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+    </row>
+    <row r="17" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="7" t="s">
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="7" t="s">
+      <c r="F17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>77</v>
       </c>
       <c r="H17" s="8" t="n">
@@ -1627,32 +1716,32 @@
         <f aca="false">B17*J17</f>
         <v>0.484</v>
       </c>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-    </row>
-    <row r="18" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+    </row>
+    <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="B18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="7" t="s">
+      <c r="F18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>82</v>
       </c>
       <c r="H18" s="8" t="n">
@@ -1669,32 +1758,32 @@
         <f aca="false">B18*J18</f>
         <v>0.369</v>
       </c>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-    </row>
-    <row r="19" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+    </row>
+    <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="7" t="s">
+      <c r="F19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>87</v>
       </c>
       <c r="H19" s="8" t="n">
@@ -1711,32 +1800,32 @@
         <f aca="false">B19*J19</f>
         <v>0.098</v>
       </c>
-      <c r="L19" s="7"/>
-      <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-    </row>
-    <row r="20" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+    </row>
+    <row r="20" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="B20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="7" t="s">
+      <c r="F20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>92</v>
       </c>
       <c r="H20" s="8" t="n">
@@ -1753,32 +1842,32 @@
         <f aca="false">B20*J20</f>
         <v>0.076</v>
       </c>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-    </row>
-    <row r="21" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+    </row>
+    <row r="21" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="7" t="s">
+      <c r="F21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>97</v>
       </c>
       <c r="H21" s="8" t="n">
@@ -1795,32 +1884,32 @@
         <f aca="false">B21*J21</f>
         <v>1.715</v>
       </c>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-    </row>
-    <row r="22" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+    </row>
+    <row r="22" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="7" t="s">
+      <c r="B22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="7" t="s">
+      <c r="F22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>101</v>
       </c>
       <c r="H22" s="8" t="n">
@@ -1837,32 +1926,32 @@
         <f aca="false">B22*J22</f>
         <v>0.045</v>
       </c>
-      <c r="L22" s="7"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-    </row>
-    <row r="23" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+    </row>
+    <row r="23" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="B23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="7" t="s">
+      <c r="F23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>106</v>
       </c>
       <c r="H23" s="8" t="n">
@@ -1879,32 +1968,32 @@
         <f aca="false">B23*J23</f>
         <v>0.342</v>
       </c>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-    </row>
-    <row r="24" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+    </row>
+    <row r="24" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="7" t="s">
+      <c r="B24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" s="7" t="s">
+      <c r="F24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>110</v>
       </c>
       <c r="H24" s="8" t="n">
@@ -1921,32 +2010,32 @@
         <f aca="false">B24*J24</f>
         <v>0.342</v>
       </c>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-    </row>
-    <row r="25" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+    </row>
+    <row r="25" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="B25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="7" t="s">
+      <c r="F25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>114</v>
       </c>
       <c r="H25" s="8" t="n">
@@ -1963,32 +2052,32 @@
         <f aca="false">B25*J25</f>
         <v>3.98</v>
       </c>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="7"/>
-    </row>
-    <row r="26" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+    </row>
+    <row r="26" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="7" t="s">
+      <c r="B26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G26" s="7" t="s">
+      <c r="F26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>119</v>
       </c>
       <c r="H26" s="8" t="n">
@@ -2005,40 +2094,40 @@
         <f aca="false">B26*J26</f>
         <v>0.38</v>
       </c>
-      <c r="L26" s="7" t="s">
+      <c r="L26" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="M26" s="7" t="s">
+      <c r="M26" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="N26" s="7" t="n">
+      <c r="N26" s="4" t="n">
         <v>0.39507</v>
       </c>
-      <c r="O26" s="7" t="n">
+      <c r="O26" s="4" t="n">
         <v>0.81</v>
       </c>
-      <c r="P26" s="7"/>
-    </row>
-    <row r="27" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="P26" s="4"/>
+    </row>
+    <row r="27" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B27" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="B27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G27" s="7" t="s">
+      <c r="F27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>126</v>
       </c>
       <c r="H27" s="8" t="n">
@@ -2055,32 +2144,32 @@
         <f aca="false">B27*J27</f>
         <v>1.31</v>
       </c>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="7"/>
-    </row>
-    <row r="28" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
+    </row>
+    <row r="28" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="7" t="s">
+      <c r="B28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G28" s="7" t="s">
+      <c r="F28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>131</v>
       </c>
       <c r="H28" s="8" t="n">
@@ -2097,32 +2186,32 @@
         <f aca="false">B28*J28</f>
         <v>2.4</v>
       </c>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-    </row>
-    <row r="29" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+    </row>
+    <row r="29" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="7" t="s">
+      <c r="B29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G29" s="7" t="s">
+      <c r="F29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>136</v>
       </c>
       <c r="H29" s="8" t="n">
@@ -2139,32 +2228,32 @@
         <f aca="false">B29*J29</f>
         <v>1.22</v>
       </c>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="7"/>
-    </row>
-    <row r="30" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
+    </row>
+    <row r="30" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G30" s="7" t="s">
+      <c r="F30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>141</v>
       </c>
       <c r="H30" s="8" t="n">
@@ -2181,32 +2270,32 @@
         <f aca="false">B30*J30</f>
         <v>0.213</v>
       </c>
-      <c r="L30" s="7"/>
-      <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="7"/>
-    </row>
-    <row r="31" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+      <c r="P30" s="4"/>
+    </row>
+    <row r="31" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="7" t="s">
+      <c r="B31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G31" s="7" t="s">
+      <c r="F31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>146</v>
       </c>
       <c r="H31" s="8" t="n">
@@ -2223,32 +2312,32 @@
         <f aca="false">B31*J31</f>
         <v>0.163</v>
       </c>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-    </row>
-    <row r="32" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+      <c r="P31" s="4"/>
+    </row>
+    <row r="32" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B32" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E32" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G32" s="7" t="s">
+      <c r="F32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="4" t="s">
         <v>150</v>
       </c>
       <c r="H32" s="8" t="n">
@@ -2265,32 +2354,32 @@
         <f aca="false">B32*J32</f>
         <v>0.398</v>
       </c>
-      <c r="L32" s="7"/>
-      <c r="M32" s="7"/>
-      <c r="N32" s="7"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="7"/>
-    </row>
-    <row r="33" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
+    </row>
+    <row r="33" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="B33" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G33" s="7" t="s">
+      <c r="F33" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="4" t="s">
         <v>155</v>
       </c>
       <c r="H33" s="8" t="n">
@@ -2307,32 +2396,32 @@
         <f aca="false">B33*J33</f>
         <v>1.818</v>
       </c>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-    </row>
-    <row r="34" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+    </row>
+    <row r="34" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="7" t="s">
+      <c r="B34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G34" s="7" t="s">
+      <c r="F34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" s="4" t="s">
         <v>160</v>
       </c>
       <c r="H34" s="8" t="n">
@@ -2349,32 +2438,32 @@
         <f aca="false">B34*J34</f>
         <v>0.42</v>
       </c>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="7"/>
-    </row>
-    <row r="35" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+    </row>
+    <row r="35" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B35" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="F35" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G35" s="7" t="s">
+      <c r="F35" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" s="4" t="s">
         <v>164</v>
       </c>
       <c r="H35" s="8" t="n">
@@ -2391,32 +2480,32 @@
         <f aca="false">B35*J35</f>
         <v>0.03</v>
       </c>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-      <c r="N35" s="7"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="7"/>
-    </row>
-    <row r="36" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+      <c r="P35" s="4"/>
+    </row>
+    <row r="36" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="B36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="7" t="s">
+      <c r="B36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G36" s="7" t="s">
+      <c r="F36" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" s="4" t="s">
         <v>168</v>
       </c>
       <c r="H36" s="8" t="n">
@@ -2433,32 +2522,32 @@
         <f aca="false">B36*J36</f>
         <v>0.021</v>
       </c>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="7"/>
-      <c r="P36" s="7"/>
-    </row>
-    <row r="37" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="4"/>
+    </row>
+    <row r="37" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="7" t="s">
+      <c r="B37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F37" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G37" s="7" t="s">
+      <c r="F37" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>173</v>
       </c>
       <c r="H37" s="8" t="n">
@@ -2475,32 +2564,32 @@
         <f aca="false">B37*J37</f>
         <v>0.043</v>
       </c>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-    </row>
-    <row r="38" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+    </row>
+    <row r="38" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="7" t="n">
+      <c r="B38" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F38" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G38" s="7" t="s">
+      <c r="F38" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="4" t="s">
         <v>177</v>
       </c>
       <c r="H38" s="8" t="n">
@@ -2517,32 +2606,32 @@
         <f aca="false">B38*J38</f>
         <v>0.372</v>
       </c>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-    </row>
-    <row r="39" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
+      <c r="P38" s="4"/>
+    </row>
+    <row r="39" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="B39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="7" t="s">
+      <c r="B39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F39" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G39" s="7" t="s">
+      <c r="F39" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39" s="4" t="s">
         <v>181</v>
       </c>
       <c r="H39" s="8" t="n">
@@ -2559,32 +2648,32 @@
         <f aca="false">B39*J39</f>
         <v>0.013</v>
       </c>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
-      <c r="P39" s="7"/>
-    </row>
-    <row r="40" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+    </row>
+    <row r="40" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B40" s="7" t="n">
+      <c r="B40" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G40" s="7" t="s">
+      <c r="F40" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" s="4" t="s">
         <v>185</v>
       </c>
       <c r="H40" s="8" t="n">
@@ -2601,32 +2690,32 @@
         <f aca="false">B40*J40</f>
         <v>0.246</v>
       </c>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
-      <c r="P40" s="7"/>
-    </row>
-    <row r="41" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+    </row>
+    <row r="41" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="7" t="s">
+      <c r="B41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F41" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G41" s="7" t="s">
+      <c r="F41" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="4" t="s">
         <v>189</v>
       </c>
       <c r="H41" s="8" t="n">
@@ -2643,32 +2732,32 @@
         <f aca="false">B41*J41</f>
         <v>0.009</v>
       </c>
-      <c r="L41" s="7"/>
-      <c r="M41" s="7"/>
-      <c r="N41" s="7"/>
-      <c r="O41" s="7"/>
-      <c r="P41" s="7"/>
-    </row>
-    <row r="42" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
+    </row>
+    <row r="42" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="7" t="s">
+      <c r="B42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="F42" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G42" s="7" t="s">
+      <c r="F42" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42" s="4" t="s">
         <v>193</v>
       </c>
       <c r="H42" s="8" t="n">
@@ -2685,32 +2774,32 @@
         <f aca="false">B42*J42</f>
         <v>0.042</v>
       </c>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-      <c r="N42" s="7"/>
-      <c r="O42" s="7"/>
-      <c r="P42" s="7"/>
-    </row>
-    <row r="43" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
+    </row>
+    <row r="43" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B43" s="7" t="n">
+      <c r="B43" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E43" s="7" t="s">
+      <c r="E43" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="F43" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G43" s="7" t="s">
+      <c r="F43" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" s="4" t="s">
         <v>197</v>
       </c>
       <c r="H43" s="8" t="n">
@@ -2727,32 +2816,32 @@
         <f aca="false">B43*J43</f>
         <v>0.062</v>
       </c>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
-      <c r="P43" s="7"/>
-    </row>
-    <row r="44" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+      <c r="P43" s="4"/>
+    </row>
+    <row r="44" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="B44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="7" t="s">
+      <c r="B44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="F44" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G44" s="7" t="s">
+      <c r="F44" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G44" s="4" t="s">
         <v>201</v>
       </c>
       <c r="H44" s="8" t="n">
@@ -2769,32 +2858,32 @@
         <f aca="false">B44*J44</f>
         <v>0.139</v>
       </c>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-      <c r="N44" s="7"/>
-      <c r="O44" s="7"/>
-      <c r="P44" s="7"/>
-    </row>
-    <row r="45" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
+    </row>
+    <row r="45" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="B45" s="7" t="n">
+      <c r="B45" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E45" s="7" t="s">
+      <c r="E45" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="F45" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G45" s="7" t="s">
+      <c r="F45" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>205</v>
       </c>
       <c r="H45" s="8" t="n">
@@ -2811,32 +2900,32 @@
         <f aca="false">B45*J45</f>
         <v>0.102</v>
       </c>
-      <c r="L45" s="7"/>
-      <c r="M45" s="7"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="7"/>
-      <c r="P45" s="7"/>
-    </row>
-    <row r="46" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+    </row>
+    <row r="46" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B46" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="7" t="s">
+      <c r="B46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="F46" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G46" s="7" t="s">
+      <c r="F46" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G46" s="4" t="s">
         <v>209</v>
       </c>
       <c r="H46" s="8" t="n">
@@ -2853,32 +2942,32 @@
         <f aca="false">B46*J46</f>
         <v>0.052</v>
       </c>
-      <c r="L46" s="7"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="7"/>
-    </row>
-    <row r="47" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+    </row>
+    <row r="47" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="7" t="s">
+      <c r="B47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="F47" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G47" s="7" t="s">
+      <c r="F47" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G47" s="4" t="s">
         <v>213</v>
       </c>
       <c r="H47" s="8" t="n">
@@ -2895,32 +2984,32 @@
         <f aca="false">B47*J47</f>
         <v>0.048</v>
       </c>
-      <c r="L47" s="7"/>
-      <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
-      <c r="P47" s="7"/>
-    </row>
-    <row r="48" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
+    </row>
+    <row r="48" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B48" s="7" t="n">
+      <c r="B48" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="D48" s="7" t="s">
+      <c r="D48" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E48" s="7" t="n">
+      <c r="E48" s="4" t="n">
         <v>435151014845</v>
       </c>
-      <c r="F48" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G48" s="7" t="s">
+      <c r="F48" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G48" s="4" t="s">
         <v>217</v>
       </c>
       <c r="H48" s="8" t="n">
@@ -2937,32 +3026,32 @@
         <f aca="false">B48*J48</f>
         <v>0.726</v>
       </c>
-      <c r="L48" s="7"/>
-      <c r="M48" s="7"/>
-      <c r="N48" s="7"/>
-      <c r="O48" s="7"/>
-      <c r="P48" s="7"/>
-    </row>
-    <row r="49" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+    </row>
+    <row r="49" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="B49" s="7" t="n">
+      <c r="B49" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C49" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="7" t="s">
+      <c r="D49" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="E49" s="7" t="n">
+      <c r="E49" s="4" t="n">
         <v>5010</v>
       </c>
-      <c r="F49" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G49" s="7" t="s">
+      <c r="F49" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G49" s="4" t="s">
         <v>221</v>
       </c>
       <c r="H49" s="8" t="n">
@@ -2979,26 +3068,26 @@
         <f aca="false">B49*J49</f>
         <v>4.324</v>
       </c>
-      <c r="L49" s="7"/>
-      <c r="M49" s="7"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="7"/>
-      <c r="P49" s="7"/>
-    </row>
-    <row r="50" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="s">
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
+    </row>
+    <row r="50" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="B50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" s="7" t="s">
+      <c r="B50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
       <c r="H50" s="8" t="n">
         <v>5</v>
       </c>
@@ -3013,32 +3102,32 @@
         <f aca="false">B50*J50</f>
         <v>1</v>
       </c>
-      <c r="L50" s="7"/>
-      <c r="M50" s="7"/>
-      <c r="N50" s="7"/>
-      <c r="O50" s="7"/>
-      <c r="P50" s="7"/>
-    </row>
-    <row r="51" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="4"/>
+    </row>
+    <row r="51" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="B51" s="7" t="n">
+      <c r="B51" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C51" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="D51" s="7" t="s">
+      <c r="D51" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="E51" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="F51" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G51" s="10" t="s">
+      <c r="F51" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>227</v>
       </c>
       <c r="H51" s="8" t="n">
@@ -3055,32 +3144,32 @@
         <f aca="false">B51*J51</f>
         <v>0.333</v>
       </c>
-      <c r="L51" s="7"/>
-      <c r="M51" s="7"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="7"/>
-      <c r="P51" s="7"/>
-    </row>
-    <row r="52" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+    </row>
+    <row r="52" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="B52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" s="7" t="s">
+      <c r="B52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="D52" s="7" t="s">
+      <c r="D52" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E52" s="7" t="s">
+      <c r="E52" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="F52" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G52" s="7" t="s">
+      <c r="F52" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" s="4" t="s">
         <v>231</v>
       </c>
       <c r="H52" s="8" t="n">
@@ -3095,32 +3184,32 @@
         <f aca="false">B52*J52</f>
         <v>0</v>
       </c>
-      <c r="L52" s="7"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7"/>
-      <c r="P52" s="7"/>
-    </row>
-    <row r="53" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+    </row>
+    <row r="53" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="B53" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="7" t="s">
+      <c r="B53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="D53" s="7" t="s">
+      <c r="D53" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E53" s="7" t="s">
+      <c r="E53" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="F53" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G53" s="7" t="s">
+      <c r="F53" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>235</v>
       </c>
       <c r="H53" s="8" t="n">
@@ -3135,32 +3224,32 @@
         <f aca="false">B53*J53</f>
         <v>0</v>
       </c>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
-      <c r="P53" s="7"/>
-    </row>
-    <row r="54" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+    </row>
+    <row r="54" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="B54" s="7" t="n">
+      <c r="B54" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D54" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="E54" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="F54" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G54" s="7" t="s">
+      <c r="F54" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" s="4" t="s">
         <v>239</v>
       </c>
       <c r="H54" s="8" t="n">
@@ -3175,32 +3264,32 @@
         <f aca="false">B54*J54</f>
         <v>0</v>
       </c>
-      <c r="L54" s="7"/>
-      <c r="M54" s="7"/>
-      <c r="N54" s="7"/>
-      <c r="O54" s="7"/>
-      <c r="P54" s="7"/>
-    </row>
-    <row r="55" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
+    </row>
+    <row r="55" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="B55" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" s="7" t="s">
+      <c r="B55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="D55" s="7" t="s">
+      <c r="D55" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E55" s="7" t="s">
+      <c r="E55" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="F55" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G55" s="10" t="s">
+      <c r="F55" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G55" s="9" t="s">
         <v>243</v>
       </c>
       <c r="H55" s="8" t="n">
@@ -3215,32 +3304,32 @@
         <f aca="false">B55*J55</f>
         <v>0</v>
       </c>
-      <c r="L55" s="7"/>
-      <c r="M55" s="7"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="7"/>
-      <c r="P55" s="7"/>
-    </row>
-    <row r="56" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
+    </row>
+    <row r="56" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B56" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="C56" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="D56" s="7" t="s">
+      <c r="D56" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E56" s="7" t="s">
+      <c r="E56" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="F56" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G56" s="10" t="s">
+      <c r="F56" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G56" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H56" s="8" t="n">
@@ -3255,32 +3344,32 @@
         <f aca="false">B56*J56</f>
         <v>0</v>
       </c>
-      <c r="L56" s="7"/>
-      <c r="M56" s="7"/>
-      <c r="N56" s="7"/>
-      <c r="O56" s="7"/>
-      <c r="P56" s="7"/>
-    </row>
-    <row r="57" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="s">
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
+    </row>
+    <row r="57" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" s="7" t="s">
+      <c r="B57" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="D57" s="7" t="s">
+      <c r="D57" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="E57" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="F57" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G57" s="10" t="s">
+      <c r="F57" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G57" s="9" t="s">
         <v>251</v>
       </c>
       <c r="H57" s="8" t="n">
@@ -3295,29 +3384,47 @@
         <f aca="false">B57*J57</f>
         <v>0</v>
       </c>
-      <c r="L57" s="7"/>
-      <c r="M57" s="7"/>
-      <c r="N57" s="7"/>
-      <c r="O57" s="7"/>
-      <c r="P57" s="7"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="6"/>
-      <c r="I58" s="6" t="n">
+      <c r="A58" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="H58" s="8" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I58" s="8" t="n">
         <f aca="false">B58*H58</f>
-        <v>0</v>
-      </c>
-      <c r="J58" s="6"/>
-      <c r="K58" s="6" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J58" s="8" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="K58" s="8" t="n">
         <f aca="false">B58*J58</f>
-        <v>0</v>
+        <v>0.541</v>
       </c>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
@@ -3326,22 +3433,40 @@
       <c r="P58" s="4"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6" t="n">
+      <c r="A59" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="I59" s="8" t="n">
         <f aca="false">B59*H59</f>
-        <v>0</v>
-      </c>
-      <c r="J59" s="6"/>
-      <c r="K59" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="J59" s="8" t="n">
+        <v>0.14975</v>
+      </c>
+      <c r="K59" s="8" t="n">
         <f aca="false">B59*J59</f>
-        <v>0</v>
+        <v>0.14975</v>
       </c>
       <c r="L59" s="4"/>
       <c r="M59" s="4"/>

</xml_diff>